<commit_message>
fix: apply 12 remaining Excel text corrections
</commit_message>
<xml_diff>
--- a/Documents/Health-RI_v2.1.0-for-FDP.xlsx
+++ b/Documents/Health-RI_v2.1.0-for-FDP.xlsx
@@ -159,7 +159,7 @@
     <t>DCAT-AP v3</t>
   </si>
   <si>
-    <t>If applicable, add URI to connected dcat:Catalog</t>
+    <t>If applicable, enter the URI of the connected dcat:Catalog.</t>
   </si>
   <si>
     <t>contact point</t>
@@ -258,7 +258,7 @@
     <t>1..n</t>
   </si>
   <si>
-    <t>Add URI to all datasets contained in this catalogue</t>
+    <t>Enter the URI for all datasets contained in this catalogue.</t>
   </si>
   <si>
     <t>description</t>
@@ -461,7 +461,7 @@
     <t>dcat:DataService</t>
   </si>
   <si>
-    <t>If applicable, add URI to dcat:DataService</t>
+    <t>If applicable, enter the URI for dcat:DataService.</t>
   </si>
   <si>
     <t>temporal coverage</t>
@@ -560,7 +560,7 @@
     <t>http://publications.europa.eu/resource/authority/access-right</t>
   </si>
   <si>
-    <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. It is foreseen that one of the three options has to be used: public, restricted, non-public.
+    <t>Information that indicates whether the Dataset is publicly accessible, has access restrictions or is not public. One of the three options must be used: public, restricted, non-public.
     Open Data (Public): The dataset is available under general open data rules, such as those covered by the High Value Datasets Implementing Regulation.
     Protected Data (Restricted): The dataset contains protected data and is accessible only under specific conditions, as outlined in regulations like the Data Governance Act.
     Sensitive Data (Non-public): The dataset includes resources that may contain sensitive or personal information, falling under regulations such as the EHDS Regulation.
@@ -579,7 +579,7 @@
     <t>healthdcatap:analytics</t>
   </si>
   <si>
-    <t>Publishers are encouraged to provide URLs pointing to document repositories where users can access or request associated resources such as technical reports of the dataset, quality measurements, usability indicators, etc. Note that HealthDCAT-AP also mentions API endpoints or analytics services, but these would not be Distributions but rather DatasetServices.</t>
+    <t>Publishers are encouraged to provide URLs pointing to document repositories where users can access or request associated resources such as technical reports of the dataset, quality measurements, usability indicators, etc. Note that HealthDCAT-AP also mentions API endpoints or analytics services, but these would be Data Services rather than Distributions.</t>
   </si>
   <si>
     <t>dcat:Distribution</t>
@@ -714,7 +714,7 @@
     <t>custom:has_version</t>
   </si>
   <si>
-    <t>fill in URI to dcat:Dataset that is another version of current Dataset</t>
+    <t>Enter the URI for the dcat:Dataset that is another version of the current Dataset.</t>
   </si>
   <si>
     <t>health theme</t>
@@ -960,7 +960,7 @@
       </rPr>
       <t xml:space="preserve">This property makes use of another small class (prov:Attribution). There, you can choose one of the roles as listed in the controlled vocabulary and link that to a specific Agent (expressed with foaf:Agent).
 Repeat this property if you wish to specify multiple roles for the same agent.
-Refer to the Attribution class for more information how to fill this.
+Refer to the Attribution class for more information on how to fill this in.
 Use this property if you would like to indicate the </t>
     </r>
     <r>
@@ -980,7 +980,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve">of the (research project that resulted in creation of the) dataset.
+      <t xml:space="preserve">of the dataset (or of the research project that resulted in its creation).
 The value for </t>
     </r>
     <r>
@@ -1627,7 +1627,7 @@
         <rFont val="Aptos Display"/>
         <scheme val="major"/>
       </rPr>
-      <t xml:space="preserve"> used in the Distribution, using a value from the EU controlled vocabulary. Not all distributions might have a language, for example imaging data.
+      <t xml:space="preserve"> used in the Distribution, using a value from the EU controlled vocabulary. Not all distributions necessarily have a language; for example, those containing imaging data may not.
 Note that here the Health-RI model diverges from DCAT-AP NL, which allows a maximum of 1 language per Distribution. The Health-RI model allows multiple languages in the same Distribution.</t>
     </r>
   </si>
@@ -2450,7 +2450,7 @@
 For example: mailto:info@example.com</t>
   </si>
   <si>
-    <t>The licence under which the catalogue (with resource description) is made available.
+    <t>The licence under which the catalogue (with its resource description) is made available.
 The licences for Distributions and Data Services are not specified here. They are specified in the licence properties of their respective classes.</t>
   </si>
   <si>
@@ -2686,7 +2686,7 @@
     <t>csvw:datatype</t>
   </si>
   <si>
-    <t>Technical variable name required to match a column header in the CSV file (synthetic, anonymized representation of the real data), can appear in multiple languages.</t>
+    <t>A technical variable name is required to match a column header in the CSV file (a synthetic, anonymised representation of the real data).</t>
   </si>
   <si>
     <t>Human-readable title(s) for the column. May be multilingual.</t>
@@ -3463,7 +3463,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Display"/>
       </rPr>
-      <t>Choose a term from the controlled vocabulary, which includes the following types: Academia-ScientificOrganisation, Company, IndustryConsortium, LocalAuthority, NationalAuthority, NonGovernmentalOrganisation, NonProfitOrganisation, PrivateIndividual, RegionalAuthority, StandardisationBody and SupraNationalAuthority. These should use the following URL: http://purl.org/adms/publishertype/[type].</t>
+      <t>Choose a term from the controlled vocabulary, which includes the following types: Academia-ScientificOrganisation, Company, IndustryConsortium, LocalAuthority, NationalAuthority, NonGovernmentalOrganisation, NonProfitOrganisation, PrivateIndividual, RegionalAuthority, StandardisationBody and SupraNationalAuthority. These should use URLs of the following form: http://purl.org/adms/publishertype/[type].</t>
     </r>
   </si>
   <si>
@@ -3514,7 +3514,8 @@
     </r>
   </si>
   <si>
-    <t>The propertyUrl may point to standard, controlled vocabularies, or ontologies that define the semantic meaning of the column. For example: csvw:propertyUrl http://publications.europa.eu/resource/authority/country For advanced usage, refer to the official specification: https://www.w3.org/TR/tabular-metadata/#propertyurl</t>
+    <t>The propertyUrl may point to standard vocabularies, controlled vocabularies or ontologies that define the semantic meaning of the column. For example: csvw:propertyUrl http://publications.europa.eu/resource/authority/country
+For advanced usage, refer to the official specification: https://www.w3.org/TR/tabular-metadata/#propertyurl</t>
   </si>
   <si>
     <t>Activity</t>

</xml_diff>